<commit_message>
actionType: bind to DesignLoad/actionType (the stale DesignAction element no longer exists)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/actionType.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/actionType.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9200" yWindow="3280" windowWidth="39400" windowHeight="24940" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lists" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -995,7 +995,7 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>//diggs:DesignAction/diggs:actionType</t>
+          <t>//diggs:DesignLoad/diggs:actionType</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>//diggs:DesignAction/diggs:actionType</t>
+          <t>//diggs:DesignLoad/diggs:actionType</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>//diggs:DesignAction/diggs:actionType</t>
+          <t>//diggs:DesignLoad/diggs:actionType</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>//diggs:DesignAction/diggs:actionType</t>
+          <t>//diggs:DesignLoad/diggs:actionType</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>//diggs:DesignAction/diggs:actionType</t>
+          <t>//diggs:DesignLoad/diggs:actionType</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>//diggs:DesignAction/diggs:actionType</t>
+          <t>//diggs:DesignLoad/diggs:actionType</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>//diggs:DesignAction/diggs:actionType</t>
+          <t>//diggs:DesignLoad/diggs:actionType</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>//diggs:DesignAction/diggs:actionType</t>
+          <t>//diggs:DesignLoad/diggs:actionType</t>
         </is>
       </c>
     </row>

</xml_diff>